<commit_message>
Đợt sửa lớn về luồng Picking, Packing, Pickup
</commit_message>
<xml_diff>
--- a/assets/packing_list.xlsx
+++ b/assets/packing_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp\htdocs\demo\s-wms\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E6204B-5EEC-4D6B-9A6F-E3FE3EBAE416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{312CF18F-C57B-4E68-9A3D-C0FE895F5ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,33 +25,51 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>invoice</t>
-  </si>
-  <si>
-    <t>case</t>
-  </si>
-  <si>
-    <t>customer</t>
-  </si>
-  <si>
-    <t>product</t>
-  </si>
-  <si>
-    <t>quantity</t>
-  </si>
-  <si>
-    <t>bucket qty</t>
-  </si>
-  <si>
-    <t>export date</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+  <si>
+    <t>Pallet No</t>
+  </si>
+  <si>
+    <t>SEA/AIR</t>
+  </si>
+  <si>
+    <t>Customer Code</t>
+  </si>
+  <si>
+    <t>Item Code</t>
+  </si>
+  <si>
+    <t>Invoice</t>
+  </si>
+  <si>
+    <t>Total Quantity</t>
+  </si>
+  <si>
+    <t>Qty.of boxes</t>
+  </si>
+  <si>
+    <t>Ngày xuất</t>
+  </si>
+  <si>
+    <t>001</t>
+  </si>
+  <si>
+    <t>11111</t>
+  </si>
+  <si>
+    <t>ABCDEFGH</t>
+  </si>
+  <si>
+    <t>VJP001</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -81,8 +99,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -363,30 +384,69 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="6.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.36328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.08984375" style="2" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="3">
+        <v>100</v>
+      </c>
+      <c r="G2" s="3">
+        <v>5</v>
+      </c>
+      <c r="H2" s="2">
+        <v>46023</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật chức năng KPI dashboard
</commit_message>
<xml_diff>
--- a/assets/packing_list.xlsx
+++ b/assets/packing_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp\htdocs\demo\s-wms\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{312CF18F-C57B-4E68-9A3D-C0FE895F5ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A935A8D-F0B7-46B9-B3C1-F9E76EC10C78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1210" yWindow="380" windowWidth="16230" windowHeight="8560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="packing_list" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>Pallet No</t>
   </si>
@@ -61,6 +61,12 @@
   </si>
   <si>
     <t>VJP001</t>
+  </si>
+  <si>
+    <t>Mã đặt hàng</t>
+  </si>
+  <si>
+    <t>ABCD-1</t>
   </si>
 </sst>
 </file>
@@ -68,7 +74,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -102,7 +108,7 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -384,7 +390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.7265625" style="1" bestFit="1" customWidth="1"/>
@@ -397,7 +403,7 @@
     <col min="8" max="8" width="10.08984375" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -422,8 +428,11 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -447,6 +456,9 @@
       </c>
       <c r="H2" s="2">
         <v>46023</v>
+      </c>
+      <c r="I2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>